<commit_message>
Marcela page: mark loan PAID IN FULL as of 7/19/2026
Final payment: Chase check #502, 2,830.71, deposited BofA Fruitville 7/21/2026 (Trans #5628). No additional interest accrued because 6/29 payment satisfied the July installment before the next accrual date. New signed/notarized acknowledgment PDF added; prior 7/16 quote letter retained. Tracker synced to zero balance.
</commit_message>
<xml_diff>
--- a/public/marcela/Marcela_Loan_Tracker.xlsx
+++ b/public/marcela/Marcela_Loan_Tracker.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="71">
   <si>
     <t xml:space="preserve">Marcela Pool Loan Tracker</t>
   </si>
@@ -224,6 +224,12 @@
   </si>
   <si>
     <t xml:space="preserve">Auto-imported. Conf# 0K788773T. Memo: Pool loan payment July 1 2026 (paid early 6/29)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAID IN FULL. Chase check #502 dated 7/19/2026, deposited BofA Fruitville Rd 7/21/2026, BofA Trans #5628. Paid before August accrual date, so no interest accrued after 6/29 payment.</t>
   </si>
   <si>
     <t xml:space="preserve">Expected Payment Schedule (84 Months, Payments Due 5th of Month)</t>
@@ -1030,7 +1036,7 @@
       </c>
       <c r="F6" s="9" t="n">
         <f aca="false">COUNT('Payment Register'!C7:C200)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1045,7 +1051,7 @@
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">C8-F6</f>
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1060,7 +1066,7 @@
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">SUMIF('Payment Register'!C7:C200,"&gt;0",'Payment Register'!D7:D200)</f>
-        <v>9893.8</v>
+        <v>52724.51</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1105,7 +1111,7 @@
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">SUMIF('Payment Register'!C7:C200,"&gt;0",'Payment Register'!G7:G200)</f>
-        <v>7169.29</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1120,7 +1126,7 @@
       </c>
       <c r="F12" s="12" t="n">
         <f aca="false">LOOKUP(2,1/('Payment Register'!H6:H200&lt;&gt;""),'Payment Register'!H6:H200)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1141,7 +1147,7 @@
       </c>
       <c r="F15" s="12" t="n">
         <f aca="false">IF(F12&lt;=0,0,IF(F7&lt;=0,F12,-PMT(C7/12,F7,F12)))</f>
-        <v>706.694261466509</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1153,7 +1159,7 @@
       </c>
       <c r="F16" s="12" t="n">
         <f aca="false">IF(F6=0,0,F12-INDEX('Expected Schedule'!G6:G89,MIN(F6,84)))</f>
-        <v>0</v>
+        <v>-42302.47</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1294,7 +1300,7 @@
       </c>
       <c r="F32" s="22" t="n">
         <f aca="false">ROUND(C34*C7/365,4)</f>
-        <v>5.8672</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1320,7 +1326,7 @@
       </c>
       <c r="C34" s="24" t="n">
         <f aca="false">F12</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="D34" s="18"/>
       <c r="E34" s="6" t="s">
@@ -1328,7 +1334,7 @@
       </c>
       <c r="F34" s="25" t="n">
         <f aca="false">IF(F33="","",C34+F33)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1345,7 +1351,7 @@
       </c>
       <c r="F35" s="24" t="n">
         <f aca="false">IF(F34="","",ROUND(F7*C12-F34,2))</f>
-        <v>6638.29</v>
+        <v>48762.3</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1909,26 +1915,33 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="35" t="str">
+      <c r="B21" s="35" t="n">
         <f aca="false">IF(C21="","",MAX($B$6:B20)+1)</f>
-        <v/>
-      </c>
-      <c r="C21" s="42"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="37" t="str">
-        <f aca="false">IF(C21="","",ROUND(H20*Dashboard!$C$7/12,2))</f>
-        <v/>
-      </c>
-      <c r="G21" s="37" t="str">
+        <v>15</v>
+      </c>
+      <c r="C21" s="36" t="n">
+        <v>46222</v>
+      </c>
+      <c r="D21" s="37" t="n">
+        <v>42830.71</v>
+      </c>
+      <c r="E21" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="F21" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="37" t="n">
         <f aca="false">IF(C21="","",IF(OR(D21="",ISBLANK(D21)),-F21,D21-F21))</f>
-        <v/>
+        <v>42830.71</v>
       </c>
       <c r="H21" s="39" t="n">
         <f aca="false">IF(C21="",H20,H20-G21)</f>
-        <v>42830.71</v>
-      </c>
-      <c r="I21" s="41"/>
+        <v>0</v>
+      </c>
+      <c r="I21" s="41" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="35" t="str">
@@ -1948,7 +1961,7 @@
       </c>
       <c r="H22" s="39" t="n">
         <f aca="false">IF(C22="",H21,H21-G22)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I22" s="41"/>
     </row>
@@ -1970,7 +1983,7 @@
       </c>
       <c r="H23" s="39" t="n">
         <f aca="false">IF(C23="",H22,H22-G23)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I23" s="41"/>
     </row>
@@ -1992,7 +2005,7 @@
       </c>
       <c r="H24" s="39" t="n">
         <f aca="false">IF(C24="",H23,H23-G24)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I24" s="41"/>
     </row>
@@ -2014,7 +2027,7 @@
       </c>
       <c r="H25" s="39" t="n">
         <f aca="false">IF(C25="",H24,H24-G25)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I25" s="41"/>
     </row>
@@ -2036,7 +2049,7 @@
       </c>
       <c r="H26" s="39" t="n">
         <f aca="false">IF(C26="",H25,H25-G26)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I26" s="41"/>
     </row>
@@ -2058,7 +2071,7 @@
       </c>
       <c r="H27" s="39" t="n">
         <f aca="false">IF(C27="",H26,H26-G27)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I27" s="41"/>
     </row>
@@ -2080,7 +2093,7 @@
       </c>
       <c r="H28" s="39" t="n">
         <f aca="false">IF(C28="",H27,H27-G28)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I28" s="41"/>
     </row>
@@ -2102,7 +2115,7 @@
       </c>
       <c r="H29" s="39" t="n">
         <f aca="false">IF(C29="",H28,H28-G29)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I29" s="41"/>
     </row>
@@ -2124,7 +2137,7 @@
       </c>
       <c r="H30" s="39" t="n">
         <f aca="false">IF(C30="",H29,H29-G30)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I30" s="41"/>
     </row>
@@ -2146,7 +2159,7 @@
       </c>
       <c r="H31" s="39" t="n">
         <f aca="false">IF(C31="",H30,H30-G31)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I31" s="41"/>
     </row>
@@ -2168,7 +2181,7 @@
       </c>
       <c r="H32" s="39" t="n">
         <f aca="false">IF(C32="",H31,H31-G32)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I32" s="41"/>
     </row>
@@ -2190,7 +2203,7 @@
       </c>
       <c r="H33" s="39" t="n">
         <f aca="false">IF(C33="",H32,H32-G33)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I33" s="41"/>
     </row>
@@ -2212,7 +2225,7 @@
       </c>
       <c r="H34" s="39" t="n">
         <f aca="false">IF(C34="",H33,H33-G34)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I34" s="41"/>
     </row>
@@ -2234,7 +2247,7 @@
       </c>
       <c r="H35" s="39" t="n">
         <f aca="false">IF(C35="",H34,H34-G35)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I35" s="41"/>
     </row>
@@ -2256,7 +2269,7 @@
       </c>
       <c r="H36" s="39" t="n">
         <f aca="false">IF(C36="",H35,H35-G36)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I36" s="41"/>
     </row>
@@ -2278,7 +2291,7 @@
       </c>
       <c r="H37" s="39" t="n">
         <f aca="false">IF(C37="",H36,H36-G37)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I37" s="41"/>
     </row>
@@ -2300,7 +2313,7 @@
       </c>
       <c r="H38" s="39" t="n">
         <f aca="false">IF(C38="",H37,H37-G38)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I38" s="41"/>
     </row>
@@ -2322,7 +2335,7 @@
       </c>
       <c r="H39" s="39" t="n">
         <f aca="false">IF(C39="",H38,H38-G39)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I39" s="41"/>
     </row>
@@ -2344,7 +2357,7 @@
       </c>
       <c r="H40" s="39" t="n">
         <f aca="false">IF(C40="",H39,H39-G40)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I40" s="41"/>
     </row>
@@ -2366,7 +2379,7 @@
       </c>
       <c r="H41" s="39" t="n">
         <f aca="false">IF(C41="",H40,H40-G41)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I41" s="41"/>
     </row>
@@ -2388,7 +2401,7 @@
       </c>
       <c r="H42" s="39" t="n">
         <f aca="false">IF(C42="",H41,H41-G42)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I42" s="41"/>
     </row>
@@ -2410,7 +2423,7 @@
       </c>
       <c r="H43" s="39" t="n">
         <f aca="false">IF(C43="",H42,H42-G43)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I43" s="41"/>
     </row>
@@ -2432,7 +2445,7 @@
       </c>
       <c r="H44" s="39" t="n">
         <f aca="false">IF(C44="",H43,H43-G44)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I44" s="41"/>
     </row>
@@ -2454,7 +2467,7 @@
       </c>
       <c r="H45" s="39" t="n">
         <f aca="false">IF(C45="",H44,H44-G45)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I45" s="41"/>
     </row>
@@ -2476,7 +2489,7 @@
       </c>
       <c r="H46" s="39" t="n">
         <f aca="false">IF(C46="",H45,H45-G46)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I46" s="41"/>
     </row>
@@ -2498,7 +2511,7 @@
       </c>
       <c r="H47" s="39" t="n">
         <f aca="false">IF(C47="",H46,H46-G47)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I47" s="41"/>
     </row>
@@ -2520,7 +2533,7 @@
       </c>
       <c r="H48" s="39" t="n">
         <f aca="false">IF(C48="",H47,H47-G48)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I48" s="41"/>
     </row>
@@ -2542,7 +2555,7 @@
       </c>
       <c r="H49" s="39" t="n">
         <f aca="false">IF(C49="",H48,H48-G49)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I49" s="41"/>
     </row>
@@ -2564,7 +2577,7 @@
       </c>
       <c r="H50" s="39" t="n">
         <f aca="false">IF(C50="",H49,H49-G50)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I50" s="41"/>
     </row>
@@ -2586,7 +2599,7 @@
       </c>
       <c r="H51" s="39" t="n">
         <f aca="false">IF(C51="",H50,H50-G51)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I51" s="41"/>
     </row>
@@ -2608,7 +2621,7 @@
       </c>
       <c r="H52" s="39" t="n">
         <f aca="false">IF(C52="",H51,H51-G52)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I52" s="41"/>
     </row>
@@ -2630,7 +2643,7 @@
       </c>
       <c r="H53" s="39" t="n">
         <f aca="false">IF(C53="",H52,H52-G53)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I53" s="41"/>
     </row>
@@ -2652,7 +2665,7 @@
       </c>
       <c r="H54" s="39" t="n">
         <f aca="false">IF(C54="",H53,H53-G54)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I54" s="41"/>
     </row>
@@ -2674,7 +2687,7 @@
       </c>
       <c r="H55" s="39" t="n">
         <f aca="false">IF(C55="",H54,H54-G55)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I55" s="41"/>
     </row>
@@ -2696,7 +2709,7 @@
       </c>
       <c r="H56" s="39" t="n">
         <f aca="false">IF(C56="",H55,H55-G56)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I56" s="41"/>
     </row>
@@ -2718,7 +2731,7 @@
       </c>
       <c r="H57" s="39" t="n">
         <f aca="false">IF(C57="",H56,H56-G57)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I57" s="41"/>
     </row>
@@ -2740,7 +2753,7 @@
       </c>
       <c r="H58" s="39" t="n">
         <f aca="false">IF(C58="",H57,H57-G58)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I58" s="41"/>
     </row>
@@ -2762,7 +2775,7 @@
       </c>
       <c r="H59" s="39" t="n">
         <f aca="false">IF(C59="",H58,H58-G59)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I59" s="41"/>
     </row>
@@ -2784,7 +2797,7 @@
       </c>
       <c r="H60" s="39" t="n">
         <f aca="false">IF(C60="",H59,H59-G60)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I60" s="41"/>
     </row>
@@ -2806,7 +2819,7 @@
       </c>
       <c r="H61" s="39" t="n">
         <f aca="false">IF(C61="",H60,H60-G61)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I61" s="41"/>
     </row>
@@ -2828,7 +2841,7 @@
       </c>
       <c r="H62" s="39" t="n">
         <f aca="false">IF(C62="",H61,H61-G62)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I62" s="41"/>
     </row>
@@ -2850,7 +2863,7 @@
       </c>
       <c r="H63" s="39" t="n">
         <f aca="false">IF(C63="",H62,H62-G63)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I63" s="41"/>
     </row>
@@ -2872,7 +2885,7 @@
       </c>
       <c r="H64" s="39" t="n">
         <f aca="false">IF(C64="",H63,H63-G64)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I64" s="41"/>
     </row>
@@ -2894,7 +2907,7 @@
       </c>
       <c r="H65" s="39" t="n">
         <f aca="false">IF(C65="",H64,H64-G65)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I65" s="41"/>
     </row>
@@ -2916,7 +2929,7 @@
       </c>
       <c r="H66" s="39" t="n">
         <f aca="false">IF(C66="",H65,H65-G66)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I66" s="41"/>
     </row>
@@ -2938,7 +2951,7 @@
       </c>
       <c r="H67" s="39" t="n">
         <f aca="false">IF(C67="",H66,H66-G67)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I67" s="41"/>
     </row>
@@ -2960,7 +2973,7 @@
       </c>
       <c r="H68" s="39" t="n">
         <f aca="false">IF(C68="",H67,H67-G68)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I68" s="41"/>
     </row>
@@ -2982,7 +2995,7 @@
       </c>
       <c r="H69" s="39" t="n">
         <f aca="false">IF(C69="",H68,H68-G69)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I69" s="41"/>
     </row>
@@ -3004,7 +3017,7 @@
       </c>
       <c r="H70" s="39" t="n">
         <f aca="false">IF(C70="",H69,H69-G70)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I70" s="41"/>
     </row>
@@ -3026,7 +3039,7 @@
       </c>
       <c r="H71" s="39" t="n">
         <f aca="false">IF(C71="",H70,H70-G71)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I71" s="41"/>
     </row>
@@ -3048,7 +3061,7 @@
       </c>
       <c r="H72" s="39" t="n">
         <f aca="false">IF(C72="",H71,H71-G72)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I72" s="41"/>
     </row>
@@ -3070,7 +3083,7 @@
       </c>
       <c r="H73" s="39" t="n">
         <f aca="false">IF(C73="",H72,H72-G73)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I73" s="41"/>
     </row>
@@ -3092,7 +3105,7 @@
       </c>
       <c r="H74" s="39" t="n">
         <f aca="false">IF(C74="",H73,H73-G74)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I74" s="41"/>
     </row>
@@ -3114,7 +3127,7 @@
       </c>
       <c r="H75" s="39" t="n">
         <f aca="false">IF(C75="",H74,H74-G75)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I75" s="41"/>
     </row>
@@ -3136,7 +3149,7 @@
       </c>
       <c r="H76" s="39" t="n">
         <f aca="false">IF(C76="",H75,H75-G76)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I76" s="41"/>
     </row>
@@ -3158,7 +3171,7 @@
       </c>
       <c r="H77" s="39" t="n">
         <f aca="false">IF(C77="",H76,H76-G77)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I77" s="41"/>
     </row>
@@ -3180,7 +3193,7 @@
       </c>
       <c r="H78" s="39" t="n">
         <f aca="false">IF(C78="",H77,H77-G78)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I78" s="41"/>
     </row>
@@ -3202,7 +3215,7 @@
       </c>
       <c r="H79" s="39" t="n">
         <f aca="false">IF(C79="",H78,H78-G79)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I79" s="41"/>
     </row>
@@ -3224,7 +3237,7 @@
       </c>
       <c r="H80" s="39" t="n">
         <f aca="false">IF(C80="",H79,H79-G80)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I80" s="41"/>
     </row>
@@ -3246,7 +3259,7 @@
       </c>
       <c r="H81" s="39" t="n">
         <f aca="false">IF(C81="",H80,H80-G81)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I81" s="41"/>
     </row>
@@ -3268,7 +3281,7 @@
       </c>
       <c r="H82" s="39" t="n">
         <f aca="false">IF(C82="",H81,H81-G82)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I82" s="41"/>
     </row>
@@ -3290,7 +3303,7 @@
       </c>
       <c r="H83" s="39" t="n">
         <f aca="false">IF(C83="",H82,H82-G83)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I83" s="41"/>
     </row>
@@ -3312,7 +3325,7 @@
       </c>
       <c r="H84" s="39" t="n">
         <f aca="false">IF(C84="",H83,H83-G84)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I84" s="41"/>
     </row>
@@ -3334,7 +3347,7 @@
       </c>
       <c r="H85" s="39" t="n">
         <f aca="false">IF(C85="",H84,H84-G85)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I85" s="41"/>
     </row>
@@ -3356,7 +3369,7 @@
       </c>
       <c r="H86" s="39" t="n">
         <f aca="false">IF(C86="",H85,H85-G86)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I86" s="41"/>
     </row>
@@ -3378,7 +3391,7 @@
       </c>
       <c r="H87" s="39" t="n">
         <f aca="false">IF(C87="",H86,H86-G87)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I87" s="41"/>
     </row>
@@ -3400,7 +3413,7 @@
       </c>
       <c r="H88" s="39" t="n">
         <f aca="false">IF(C88="",H87,H87-G88)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I88" s="41"/>
     </row>
@@ -3422,7 +3435,7 @@
       </c>
       <c r="H89" s="39" t="n">
         <f aca="false">IF(C89="",H88,H88-G89)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I89" s="41"/>
     </row>
@@ -3444,7 +3457,7 @@
       </c>
       <c r="H90" s="39" t="n">
         <f aca="false">IF(C90="",H89,H89-G90)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I90" s="41"/>
     </row>
@@ -3466,7 +3479,7 @@
       </c>
       <c r="H91" s="39" t="n">
         <f aca="false">IF(C91="",H90,H90-G91)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I91" s="41"/>
     </row>
@@ -3488,7 +3501,7 @@
       </c>
       <c r="H92" s="39" t="n">
         <f aca="false">IF(C92="",H91,H91-G92)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I92" s="41"/>
     </row>
@@ -3510,7 +3523,7 @@
       </c>
       <c r="H93" s="39" t="n">
         <f aca="false">IF(C93="",H92,H92-G93)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I93" s="41"/>
     </row>
@@ -3532,7 +3545,7 @@
       </c>
       <c r="H94" s="39" t="n">
         <f aca="false">IF(C94="",H93,H93-G94)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I94" s="41"/>
     </row>
@@ -3554,7 +3567,7 @@
       </c>
       <c r="H95" s="39" t="n">
         <f aca="false">IF(C95="",H94,H94-G95)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I95" s="41"/>
     </row>
@@ -3576,7 +3589,7 @@
       </c>
       <c r="H96" s="39" t="n">
         <f aca="false">IF(C96="",H95,H95-G96)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I96" s="41"/>
     </row>
@@ -3598,7 +3611,7 @@
       </c>
       <c r="H97" s="39" t="n">
         <f aca="false">IF(C97="",H96,H96-G97)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I97" s="41"/>
     </row>
@@ -3620,7 +3633,7 @@
       </c>
       <c r="H98" s="39" t="n">
         <f aca="false">IF(C98="",H97,H97-G98)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I98" s="41"/>
     </row>
@@ -3642,7 +3655,7 @@
       </c>
       <c r="H99" s="39" t="n">
         <f aca="false">IF(C99="",H98,H98-G99)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I99" s="41"/>
     </row>
@@ -3664,7 +3677,7 @@
       </c>
       <c r="H100" s="39" t="n">
         <f aca="false">IF(C100="",H99,H99-G100)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
       <c r="I100" s="41"/>
     </row>
@@ -3683,7 +3696,7 @@
       </c>
       <c r="H101" s="43" t="n">
         <f aca="false">IF(C101="",H100,H100-G101)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3701,7 +3714,7 @@
       </c>
       <c r="H102" s="43" t="n">
         <f aca="false">IF(C102="",H101,H101-G102)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3719,7 +3732,7 @@
       </c>
       <c r="H103" s="43" t="n">
         <f aca="false">IF(C103="",H102,H102-G103)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3737,7 +3750,7 @@
       </c>
       <c r="H104" s="43" t="n">
         <f aca="false">IF(C104="",H103,H103-G104)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3755,7 +3768,7 @@
       </c>
       <c r="H105" s="43" t="n">
         <f aca="false">IF(C105="",H104,H104-G105)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3773,7 +3786,7 @@
       </c>
       <c r="H106" s="43" t="n">
         <f aca="false">IF(C106="",H105,H105-G106)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3791,7 +3804,7 @@
       </c>
       <c r="H107" s="43" t="n">
         <f aca="false">IF(C107="",H106,H106-G107)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3809,7 +3822,7 @@
       </c>
       <c r="H108" s="43" t="n">
         <f aca="false">IF(C108="",H107,H107-G108)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3827,7 +3840,7 @@
       </c>
       <c r="H109" s="43" t="n">
         <f aca="false">IF(C109="",H108,H108-G109)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3845,7 +3858,7 @@
       </c>
       <c r="H110" s="43" t="n">
         <f aca="false">IF(C110="",H109,H109-G110)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3863,7 +3876,7 @@
       </c>
       <c r="H111" s="43" t="n">
         <f aca="false">IF(C111="",H110,H110-G111)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3881,7 +3894,7 @@
       </c>
       <c r="H112" s="43" t="n">
         <f aca="false">IF(C112="",H111,H111-G112)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3899,7 +3912,7 @@
       </c>
       <c r="H113" s="43" t="n">
         <f aca="false">IF(C113="",H112,H112-G113)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3917,7 +3930,7 @@
       </c>
       <c r="H114" s="43" t="n">
         <f aca="false">IF(C114="",H113,H113-G114)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3935,7 +3948,7 @@
       </c>
       <c r="H115" s="43" t="n">
         <f aca="false">IF(C115="",H114,H114-G115)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3953,7 +3966,7 @@
       </c>
       <c r="H116" s="43" t="n">
         <f aca="false">IF(C116="",H115,H115-G116)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3971,7 +3984,7 @@
       </c>
       <c r="H117" s="43" t="n">
         <f aca="false">IF(C117="",H116,H116-G117)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3989,7 +4002,7 @@
       </c>
       <c r="H118" s="43" t="n">
         <f aca="false">IF(C118="",H117,H117-G118)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4007,7 +4020,7 @@
       </c>
       <c r="H119" s="43" t="n">
         <f aca="false">IF(C119="",H118,H118-G119)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4025,7 +4038,7 @@
       </c>
       <c r="H120" s="43" t="n">
         <f aca="false">IF(C120="",H119,H119-G120)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4043,7 +4056,7 @@
       </c>
       <c r="H121" s="43" t="n">
         <f aca="false">IF(C121="",H120,H120-G121)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4061,7 +4074,7 @@
       </c>
       <c r="H122" s="43" t="n">
         <f aca="false">IF(C122="",H121,H121-G122)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4079,7 +4092,7 @@
       </c>
       <c r="H123" s="43" t="n">
         <f aca="false">IF(C123="",H122,H122-G123)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4097,7 +4110,7 @@
       </c>
       <c r="H124" s="43" t="n">
         <f aca="false">IF(C124="",H123,H123-G124)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4115,7 +4128,7 @@
       </c>
       <c r="H125" s="43" t="n">
         <f aca="false">IF(C125="",H124,H124-G125)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4133,7 +4146,7 @@
       </c>
       <c r="H126" s="43" t="n">
         <f aca="false">IF(C126="",H125,H125-G126)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4151,7 +4164,7 @@
       </c>
       <c r="H127" s="43" t="n">
         <f aca="false">IF(C127="",H126,H126-G127)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4169,7 +4182,7 @@
       </c>
       <c r="H128" s="43" t="n">
         <f aca="false">IF(C128="",H127,H127-G128)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4187,7 +4200,7 @@
       </c>
       <c r="H129" s="43" t="n">
         <f aca="false">IF(C129="",H128,H128-G129)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4205,7 +4218,7 @@
       </c>
       <c r="H130" s="43" t="n">
         <f aca="false">IF(C130="",H129,H129-G130)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4223,7 +4236,7 @@
       </c>
       <c r="H131" s="43" t="n">
         <f aca="false">IF(C131="",H130,H130-G131)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4241,7 +4254,7 @@
       </c>
       <c r="H132" s="43" t="n">
         <f aca="false">IF(C132="",H131,H131-G132)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4259,7 +4272,7 @@
       </c>
       <c r="H133" s="43" t="n">
         <f aca="false">IF(C133="",H132,H132-G133)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4277,7 +4290,7 @@
       </c>
       <c r="H134" s="43" t="n">
         <f aca="false">IF(C134="",H133,H133-G134)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4295,7 +4308,7 @@
       </c>
       <c r="H135" s="43" t="n">
         <f aca="false">IF(C135="",H134,H134-G135)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4313,7 +4326,7 @@
       </c>
       <c r="H136" s="43" t="n">
         <f aca="false">IF(C136="",H135,H135-G136)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4331,7 +4344,7 @@
       </c>
       <c r="H137" s="43" t="n">
         <f aca="false">IF(C137="",H136,H136-G137)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4349,7 +4362,7 @@
       </c>
       <c r="H138" s="43" t="n">
         <f aca="false">IF(C138="",H137,H137-G138)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4367,7 +4380,7 @@
       </c>
       <c r="H139" s="43" t="n">
         <f aca="false">IF(C139="",H138,H138-G139)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4385,7 +4398,7 @@
       </c>
       <c r="H140" s="43" t="n">
         <f aca="false">IF(C140="",H139,H139-G140)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4403,7 +4416,7 @@
       </c>
       <c r="H141" s="43" t="n">
         <f aca="false">IF(C141="",H140,H140-G141)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4421,7 +4434,7 @@
       </c>
       <c r="H142" s="43" t="n">
         <f aca="false">IF(C142="",H141,H141-G142)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4439,7 +4452,7 @@
       </c>
       <c r="H143" s="43" t="n">
         <f aca="false">IF(C143="",H142,H142-G143)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4457,7 +4470,7 @@
       </c>
       <c r="H144" s="43" t="n">
         <f aca="false">IF(C144="",H143,H143-G144)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4475,7 +4488,7 @@
       </c>
       <c r="H145" s="43" t="n">
         <f aca="false">IF(C145="",H144,H144-G145)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4493,7 +4506,7 @@
       </c>
       <c r="H146" s="43" t="n">
         <f aca="false">IF(C146="",H145,H145-G146)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4511,7 +4524,7 @@
       </c>
       <c r="H147" s="43" t="n">
         <f aca="false">IF(C147="",H146,H146-G147)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4529,7 +4542,7 @@
       </c>
       <c r="H148" s="43" t="n">
         <f aca="false">IF(C148="",H147,H147-G148)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4547,7 +4560,7 @@
       </c>
       <c r="H149" s="43" t="n">
         <f aca="false">IF(C149="",H148,H148-G149)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4565,7 +4578,7 @@
       </c>
       <c r="H150" s="43" t="n">
         <f aca="false">IF(C150="",H149,H149-G150)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4583,7 +4596,7 @@
       </c>
       <c r="H151" s="43" t="n">
         <f aca="false">IF(C151="",H150,H150-G151)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4601,7 +4614,7 @@
       </c>
       <c r="H152" s="43" t="n">
         <f aca="false">IF(C152="",H151,H151-G152)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4619,7 +4632,7 @@
       </c>
       <c r="H153" s="43" t="n">
         <f aca="false">IF(C153="",H152,H152-G153)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4637,7 +4650,7 @@
       </c>
       <c r="H154" s="43" t="n">
         <f aca="false">IF(C154="",H153,H153-G154)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4655,7 +4668,7 @@
       </c>
       <c r="H155" s="43" t="n">
         <f aca="false">IF(C155="",H154,H154-G155)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4673,7 +4686,7 @@
       </c>
       <c r="H156" s="43" t="n">
         <f aca="false">IF(C156="",H155,H155-G156)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4691,7 +4704,7 @@
       </c>
       <c r="H157" s="43" t="n">
         <f aca="false">IF(C157="",H156,H156-G157)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4709,7 +4722,7 @@
       </c>
       <c r="H158" s="43" t="n">
         <f aca="false">IF(C158="",H157,H157-G158)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4727,7 +4740,7 @@
       </c>
       <c r="H159" s="43" t="n">
         <f aca="false">IF(C159="",H158,H158-G159)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4745,7 +4758,7 @@
       </c>
       <c r="H160" s="43" t="n">
         <f aca="false">IF(C160="",H159,H159-G160)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4763,7 +4776,7 @@
       </c>
       <c r="H161" s="43" t="n">
         <f aca="false">IF(C161="",H160,H160-G161)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4781,7 +4794,7 @@
       </c>
       <c r="H162" s="43" t="n">
         <f aca="false">IF(C162="",H161,H161-G162)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4799,7 +4812,7 @@
       </c>
       <c r="H163" s="43" t="n">
         <f aca="false">IF(C163="",H162,H162-G163)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4817,7 +4830,7 @@
       </c>
       <c r="H164" s="43" t="n">
         <f aca="false">IF(C164="",H163,H163-G164)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4835,7 +4848,7 @@
       </c>
       <c r="H165" s="43" t="n">
         <f aca="false">IF(C165="",H164,H164-G165)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4853,7 +4866,7 @@
       </c>
       <c r="H166" s="43" t="n">
         <f aca="false">IF(C166="",H165,H165-G166)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4871,7 +4884,7 @@
       </c>
       <c r="H167" s="43" t="n">
         <f aca="false">IF(C167="",H166,H166-G167)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4889,7 +4902,7 @@
       </c>
       <c r="H168" s="43" t="n">
         <f aca="false">IF(C168="",H167,H167-G168)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4907,7 +4920,7 @@
       </c>
       <c r="H169" s="43" t="n">
         <f aca="false">IF(C169="",H168,H168-G169)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4925,7 +4938,7 @@
       </c>
       <c r="H170" s="43" t="n">
         <f aca="false">IF(C170="",H169,H169-G170)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4943,7 +4956,7 @@
       </c>
       <c r="H171" s="43" t="n">
         <f aca="false">IF(C171="",H170,H170-G171)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4961,7 +4974,7 @@
       </c>
       <c r="H172" s="43" t="n">
         <f aca="false">IF(C172="",H171,H171-G172)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4979,7 +4992,7 @@
       </c>
       <c r="H173" s="43" t="n">
         <f aca="false">IF(C173="",H172,H172-G173)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4997,7 +5010,7 @@
       </c>
       <c r="H174" s="43" t="n">
         <f aca="false">IF(C174="",H173,H173-G174)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5015,7 +5028,7 @@
       </c>
       <c r="H175" s="43" t="n">
         <f aca="false">IF(C175="",H174,H174-G175)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5033,7 +5046,7 @@
       </c>
       <c r="H176" s="43" t="n">
         <f aca="false">IF(C176="",H175,H175-G176)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5051,7 +5064,7 @@
       </c>
       <c r="H177" s="43" t="n">
         <f aca="false">IF(C177="",H176,H176-G177)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5069,7 +5082,7 @@
       </c>
       <c r="H178" s="43" t="n">
         <f aca="false">IF(C178="",H177,H177-G178)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5087,7 +5100,7 @@
       </c>
       <c r="H179" s="43" t="n">
         <f aca="false">IF(C179="",H178,H178-G179)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5105,7 +5118,7 @@
       </c>
       <c r="H180" s="43" t="n">
         <f aca="false">IF(C180="",H179,H179-G180)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5123,7 +5136,7 @@
       </c>
       <c r="H181" s="43" t="n">
         <f aca="false">IF(C181="",H180,H180-G181)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5141,7 +5154,7 @@
       </c>
       <c r="H182" s="43" t="n">
         <f aca="false">IF(C182="",H181,H181-G182)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5159,7 +5172,7 @@
       </c>
       <c r="H183" s="43" t="n">
         <f aca="false">IF(C183="",H182,H182-G183)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5177,7 +5190,7 @@
       </c>
       <c r="H184" s="43" t="n">
         <f aca="false">IF(C184="",H183,H183-G184)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5195,7 +5208,7 @@
       </c>
       <c r="H185" s="43" t="n">
         <f aca="false">IF(C185="",H184,H184-G185)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5213,7 +5226,7 @@
       </c>
       <c r="H186" s="43" t="n">
         <f aca="false">IF(C186="",H185,H185-G186)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5231,7 +5244,7 @@
       </c>
       <c r="H187" s="43" t="n">
         <f aca="false">IF(C187="",H186,H186-G187)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5249,7 +5262,7 @@
       </c>
       <c r="H188" s="43" t="n">
         <f aca="false">IF(C188="",H187,H187-G188)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5267,7 +5280,7 @@
       </c>
       <c r="H189" s="43" t="n">
         <f aca="false">IF(C189="",H188,H188-G189)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5285,7 +5298,7 @@
       </c>
       <c r="H190" s="43" t="n">
         <f aca="false">IF(C190="",H189,H189-G190)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5303,7 +5316,7 @@
       </c>
       <c r="H191" s="43" t="n">
         <f aca="false">IF(C191="",H190,H190-G191)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5321,7 +5334,7 @@
       </c>
       <c r="H192" s="43" t="n">
         <f aca="false">IF(C192="",H191,H191-G192)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5339,7 +5352,7 @@
       </c>
       <c r="H193" s="43" t="n">
         <f aca="false">IF(C193="",H192,H192-G193)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5357,7 +5370,7 @@
       </c>
       <c r="H194" s="43" t="n">
         <f aca="false">IF(C194="",H193,H193-G194)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5375,7 +5388,7 @@
       </c>
       <c r="H195" s="43" t="n">
         <f aca="false">IF(C195="",H194,H194-G195)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5393,7 +5406,7 @@
       </c>
       <c r="H196" s="43" t="n">
         <f aca="false">IF(C196="",H195,H195-G196)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5411,7 +5424,7 @@
       </c>
       <c r="H197" s="43" t="n">
         <f aca="false">IF(C197="",H196,H196-G197)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5429,7 +5442,7 @@
       </c>
       <c r="H198" s="43" t="n">
         <f aca="false">IF(C198="",H197,H197-G198)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5447,7 +5460,7 @@
       </c>
       <c r="H199" s="43" t="n">
         <f aca="false">IF(C199="",H198,H198-G199)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5465,7 +5478,7 @@
       </c>
       <c r="H200" s="43" t="n">
         <f aca="false">IF(C200="",H199,H199-G200)</f>
-        <v>42830.71</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5524,7 +5537,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="28" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C2" s="28"/>
       <c r="D2" s="28"/>
@@ -5534,7 +5547,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -5550,7 +5563,7 @@
         <v>42</v>
       </c>
       <c r="D5" s="44" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>45</v>

</xml_diff>